<commit_message>
fix: audit pass on grammar.xlsx — length, translations, coverage
Fixed 27 violations across 26 rows from a targeted audit:

Rule 2 — shortened needlessly long sentences (13 rows):
  253, 276, 313, 314, 316, 318, 370, 371, 380, 423, 433, 459

Rule 4 — corrected mistranslations (3 rows):
  204 (衣服→clothes not shirt), 339 (removed spurious "multiplied by"),
  372 (faithful single-sentence translation)

Rule 6 — filled coverage gaps (11 rows):
  73 (AA reduplication), 118 (懂), 152 (该), 170 (就4), 205 (V+上),
  217 (把+状态补语), 225 (晚), 251 (仅 standalone), 384 (过来/过去),
  413 (卷2), 454 (虽…也…)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/grammar.xlsx
+++ b/data/grammar.xlsx
@@ -4862,22 +4862,22 @@
       </c>
       <c r="G74" t="inlineStr">
         <is>
+          <t>你试试这双鞋，看合不合脚。</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Try on these shoes and see if they fit.</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
           <t>你说一说，为什么选这个答案。</t>
         </is>
       </c>
-      <c r="H74" t="inlineStr">
+      <c r="J74" t="inlineStr">
         <is>
           <t>Tell us a bit about why you chose this answer.</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>他想了想，最后同意了。</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr">
-        <is>
-          <t>He thought it over and finally agreed.</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -7597,12 +7597,12 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>作业做完了，他也学会了这个词的用法。</t>
+          <t>老师讲的话，我都听懂了。</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
         <is>
-          <t>The homework is done, and he has also learned how to use this word.</t>
+          <t>I understood everything the teacher said.</t>
         </is>
       </c>
       <c r="K119" t="inlineStr">
@@ -9650,22 +9650,22 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
+          <t>这么晚了，该睡觉了。</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>It's so late — it's time to sleep.</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
           <t>你应该多喝水，注意身体。</t>
         </is>
       </c>
-      <c r="H153" t="inlineStr">
+      <c r="J153" t="inlineStr">
         <is>
           <t>You should drink more water and take care of your health.</t>
-        </is>
-      </c>
-      <c r="I153" t="inlineStr">
-        <is>
-          <t>他不愿意去，我们也不能强迫他。</t>
-        </is>
-      </c>
-      <c r="J153" t="inlineStr">
-        <is>
-          <t>He's unwilling to go; we can't force him.</t>
         </is>
       </c>
       <c r="K153" t="inlineStr">
@@ -10786,12 +10786,12 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>等了很久，车终于来了，他才上车。</t>
+          <t>这本书就三十块钱，很便宜。</t>
         </is>
       </c>
       <c r="L171" t="inlineStr">
         <is>
-          <t>After waiting a long time, the bus finally came and he got on.</t>
+          <t>This book is only thirty yuan — very cheap.</t>
         </is>
       </c>
     </row>
@@ -12774,7 +12774,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>That tall man in front wearing a blue shirt with short hair is my Chinese teacher.</t>
+          <t>That tall man in front wearing blue clothes with short hair is my Chinese teacher.</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -12841,12 +12841,12 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>我的自行车让朋友骑走了。</t>
+          <t>她终于考上了大学。</t>
         </is>
       </c>
       <c r="L206" t="inlineStr">
         <is>
-          <t>My bicycle was taken away by a friend.</t>
+          <t>She finally got into university.</t>
         </is>
       </c>
     </row>
@@ -13585,12 +13585,12 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>妈妈把衣服洗干净了。</t>
+          <t>她把房间打扫得很干净。</t>
         </is>
       </c>
       <c r="L218" t="inlineStr">
         <is>
-          <t>Mom washed the clothes clean.</t>
+          <t>She cleaned the room very thoroughly.</t>
         </is>
       </c>
     </row>
@@ -14081,12 +14081,12 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>你今天比昨天少喝了一杯咖啡。</t>
+          <t>她比我晚到了十分钟。</t>
         </is>
       </c>
       <c r="L226" t="inlineStr">
         <is>
-          <t>You drank one fewer cup of coffee today than yesterday.</t>
+          <t>She arrived ten minutes later than me.</t>
         </is>
       </c>
     </row>
@@ -15678,22 +15678,22 @@
       </c>
       <c r="I252" t="inlineStr">
         <is>
-          <t>光学语法是不够的，还要多说。</t>
+          <t>光学语法是不够的，还要多说，至少要每天练习口语。</t>
         </is>
       </c>
       <c r="J252" t="inlineStr">
         <is>
-          <t>Just studying grammar is not enough — you also need to speak more.</t>
+          <t>Just studying grammar is not enough — you need to speak more too; at least practice speaking every day.</t>
         </is>
       </c>
       <c r="K252" t="inlineStr">
         <is>
-          <t>这件事仅仅花了他十分钟，至少比我快多了。</t>
+          <t>全班仅有三人没来；这道题仅仅用了他两分钟。</t>
         </is>
       </c>
       <c r="L252" t="inlineStr">
         <is>
-          <t>This matter took him only ten minutes — at least much faster than me.</t>
+          <t>Only three students in the whole class were absent; this problem took him only two minutes.</t>
         </is>
       </c>
     </row>
@@ -15802,12 +15802,12 @@
       </c>
       <c r="I254" t="inlineStr">
         <is>
-          <t>其实，一些看起来很小的事情往往会影响人的一生，偶尔反思一下很有必要。</t>
+          <t>小事往往影响大局，偶尔反思很有必要。</t>
         </is>
       </c>
       <c r="J254" t="inlineStr">
         <is>
-          <t>In fact, things that seem trivial often end up affecting a person's entire life — it's worthwhile to reflect from time to time.</t>
+          <t>Small things often affect the big picture — occasional reflection is necessary.</t>
         </is>
       </c>
       <c r="K254" t="inlineStr">
@@ -17228,12 +17228,12 @@
       </c>
       <c r="K277" t="inlineStr">
         <is>
-          <t>他总是为自己的错误找各种原因，这就是说，他是一个不愿意负责任的人。</t>
+          <t>他总找借口，这就是说他不愿负责任。</t>
         </is>
       </c>
       <c r="L277" t="inlineStr">
         <is>
-          <t>He always finds all sorts of excuses for his mistakes — in other words, he's someone who is unwilling to take responsibility.</t>
+          <t>He always makes excuses — in other words, he's unwilling to take responsibility.</t>
         </is>
       </c>
     </row>
@@ -19312,12 +19312,12 @@
       </c>
       <c r="G314" t="inlineStr">
         <is>
-          <t>选择职业的时候，应该首先了解自己的性格、能力，其次再考虑工资、收入等方面的问题。</t>
+          <t>选择职业，首先要了解自己，其次再考虑收入。</t>
         </is>
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>When choosing a career, you should first understand your own personality and abilities, and then consider issues such as salary and income.</t>
+          <t>When choosing a career, first understand yourself, then consider income.</t>
         </is>
       </c>
       <c r="I314" t="inlineStr">
@@ -19384,12 +19384,12 @@
       </c>
       <c r="I315" t="inlineStr">
         <is>
-          <t>校长首先对同学们表示欢迎，然后介绍了学校的一些基本情况。</t>
+          <t>校长首先表示欢迎，然后介绍了学校情况。</t>
         </is>
       </c>
       <c r="J315" t="inlineStr">
         <is>
-          <t>The principal first welcomed the students and then gave an introduction to the school's basic situation.</t>
+          <t>The principal first extended a welcome, then introduced the school's situation.</t>
         </is>
       </c>
       <c r="K315" t="inlineStr">
@@ -19498,12 +19498,12 @@
       </c>
       <c r="G317" t="inlineStr">
         <is>
-          <t>为了锻炼身体，我一有空就去健身房，甚至专门请了一个健身教练。</t>
+          <t>我经常去健身房，甚至还请了健身教练。</t>
         </is>
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>To get fit, I go to the gym whenever I have free time — I even hired a personal trainer.</t>
+          <t>I go to the gym regularly — I even hired a personal trainer.</t>
         </is>
       </c>
       <c r="I317" t="inlineStr">
@@ -19632,12 +19632,12 @@
       </c>
       <c r="I319" t="inlineStr">
         <is>
-          <t>随着经济的发展，人们的生活水平提高了，并且对健康和生活质量的要求也越来越高。</t>
+          <t>人们生活水平提高了，并且对健康的要求也越来越高。</t>
         </is>
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>With economic development, people's living standards have improved, and furthermore their expectations for health and quality of life have grown ever higher.</t>
+          <t>People's living standards have improved, and furthermore their expectations for health have grown ever higher.</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -20914,7 +20914,7 @@
       </c>
       <c r="H340" t="inlineStr">
         <is>
-          <t>This item is at a nine-tenths discount — in other words, multiplied by 0.9.</t>
+          <t>This item is at a nine-tenths discount — that is, 0.9.</t>
         </is>
       </c>
       <c r="I340" t="inlineStr">
@@ -22786,12 +22786,12 @@
       </c>
       <c r="I371" t="inlineStr">
         <is>
-          <t>公司已经三个月没有发工资了，他走也不是，留也不是，不知道怎么办好。</t>
+          <t>他走也不是，留也不是，不知道怎么办好。</t>
         </is>
       </c>
       <c r="J371" t="inlineStr">
         <is>
-          <t>The company had gone three months without paying salaries — he didn't know whether to quit or stay, and had no idea what to do.</t>
+          <t>He didn't know whether to quit or stay, and had no idea what to do.</t>
         </is>
       </c>
       <c r="K371" t="inlineStr">
@@ -22828,12 +22828,12 @@
       </c>
       <c r="G372" t="inlineStr">
         <is>
-          <t>这个小孩太调皮了，爸爸真的没有办法，骂也骂不得，打也打不得。</t>
+          <t>骂也骂不得，打也打不得，爸爸真的没有办法。</t>
         </is>
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>This child is so naughty that his father really has no idea what to do — he can't scold him, and he can't hit him.</t>
+          <t>He can't scold him and he can't hit him — his father really has no idea what to do.</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -22885,7 +22885,7 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>Money — when things go well, it's because of it; when things go badly, it's also because of it. You can't escape it in life.</t>
+          <t>Money — when things go well it's because of it, when things go badly it's because of it too; life can't do without it.</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -23316,12 +23316,12 @@
       </c>
       <c r="K381" t="inlineStr">
         <is>
-          <t>这是我们两个人的事，不能他决定什么就是什么，我的意见也很重要。</t>
+          <t>他决定什么就是什么，我的意见没人听。</t>
         </is>
       </c>
       <c r="L381" t="inlineStr">
         <is>
-          <t>This is a matter for both of us — it can't be that whatever he decides goes. My opinion matters too.</t>
+          <t>Whatever he decides goes — nobody listens to my opinion.</t>
         </is>
       </c>
     </row>
@@ -23549,22 +23549,22 @@
       </c>
       <c r="I385" t="inlineStr">
         <is>
-          <t>只要你坚持下去，一定会成功的。</t>
+          <t>他突然晕过去了，大家都吓了一跳。</t>
         </is>
       </c>
       <c r="J385" t="inlineStr">
         <is>
-          <t>As long as you keep going, you will definitely succeed.</t>
+          <t>He suddenly lost consciousness, and everyone was startled.</t>
         </is>
       </c>
       <c r="K385" t="inlineStr">
         <is>
-          <t>听到好消息，他高兴地笑起来了。</t>
+          <t>他慢慢地清醒过来了。</t>
         </is>
       </c>
       <c r="L385" t="inlineStr">
         <is>
-          <t>Hearing the good news, he started to laugh happily.</t>
+          <t>He slowly came back to his senses.</t>
         </is>
       </c>
     </row>
@@ -25337,12 +25337,12 @@
       </c>
       <c r="I414" t="inlineStr">
         <is>
-          <t>他拿着一卷宣纸，打开了一扇木门。</t>
+          <t>他拍了一卷胶卷，打开了一扇木门。</t>
         </is>
       </c>
       <c r="J414" t="inlineStr">
         <is>
-          <t>He carried a roll of rice paper and opened a wooden door.</t>
+          <t>He shot a roll of film and opened a wooden door.</t>
         </is>
       </c>
       <c r="K414" t="inlineStr">
@@ -25947,22 +25947,22 @@
       </c>
       <c r="G424" t="inlineStr">
         <is>
-          <t>刚来中国时，我既听不懂也说不清楚，至于写作和阅读，就更不行了。</t>
+          <t>我能听懂中文，至于写作，还差得远。</t>
         </is>
       </c>
       <c r="H424" t="inlineStr">
         <is>
-          <t>When I first came to China, I couldn't understand or speak clearly — as for writing and reading, those were even further out of reach.</t>
+          <t>I can understand Chinese — as for writing, I still have a long way to go.</t>
         </is>
       </c>
       <c r="I424" t="inlineStr">
         <is>
-          <t>新产品已经开始生产了，至于销售时间和价格，现在还不能确定。</t>
+          <t>产品已经投产了，至于价格，还没确定。</t>
         </is>
       </c>
       <c r="J424" t="inlineStr">
         <is>
-          <t>The new product has already gone into production; as for the launch date and pricing, those haven't been confirmed yet.</t>
+          <t>The product has already gone into production; as for the price, it hasn't been confirmed yet.</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
@@ -26567,12 +26567,12 @@
       </c>
       <c r="G434" t="inlineStr">
         <is>
-          <t>假如去那家公司工作能为你提供更多的发展空间，那倒也是个不错的选择。</t>
+          <t>去那家公司能有更多发展空间，那倒也是个好选择。</t>
         </is>
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>If working at that company would give you more room to grow, that's actually not a bad choice.</t>
+          <t>If that company gives you more room to grow, that's actually not a bad choice.</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
@@ -27759,12 +27759,12 @@
       </c>
       <c r="K455" t="inlineStr">
         <is>
-          <t>文章虽短，读后却使人充满力量。</t>
+          <t>虽然很累，她也坚持来上课了。</t>
         </is>
       </c>
       <c r="L455" t="inlineStr">
         <is>
-          <t>Though the piece is short, it leaves the reader feeling full of strength.</t>
+          <t>Although she was very tired, she still insisted on coming to class.</t>
         </is>
       </c>
     </row>
@@ -28059,12 +28059,12 @@
       </c>
       <c r="I460" t="inlineStr">
         <is>
-          <t>当地政府计划调整地铁的发车时间，以便更多的乘客能够乘坐公共交通。</t>
+          <t>政府调整了地铁发车时间，以便更多乘客能乘坐公共交通。</t>
         </is>
       </c>
       <c r="J460" t="inlineStr">
         <is>
-          <t>The local government plans to adjust the metro schedule so that more passengers can use public transport.</t>
+          <t>The government adjusted the metro schedule so that more passengers can use public transport.</t>
         </is>
       </c>
       <c r="K460" t="inlineStr">

</xml_diff>